<commit_message>
Macherpfote: Startklar-Fahrplan Echt jetzt!, Korrekturen Drehtage und Messbogen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Emp5GxKSE7qucfjnqnS37G
</commit_message>
<xml_diff>
--- a/pottpic-team/analyse/2026-10-30-echt-jetzt-messbogen.xlsx
+++ b/pottpic-team/analyse/2026-10-30-echt-jetzt-messbogen.xlsx
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -120,14 +119,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,7 +138,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -151,8 +150,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,12 +612,12 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>46356</v>
+      <c r="A5" s="16" t="n">
+        <v>46328</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Startwert: 16.11.–29.11.2026 (vor dem Start messen, Mo vormittags)</t>
+          <t>Startwert: 19.10.–01.11.2026 (vor dem ersten Teaser am 05.11.; ab Mo 02.11. über benutzerdefinierten Zeitraum ablesen)</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -622,10 +628,14 @@
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
-      <c r="K5" s="7" t="n"/>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Korrektur 30.10. (Macherpfote): Startwert vor den Teasern gemessen, Weihnachts-Minis finden nicht statt. Newsletter-Startwert = 0.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="17" t="n">
         <v>46370</v>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -644,7 +654,7 @@
       <c r="K6" s="7" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="17" t="n">
         <v>46384</v>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -663,7 +673,7 @@
       <c r="K7" s="7" t="n"/>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="17" t="n">
         <v>46398</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -682,7 +692,7 @@
       <c r="K8" s="7" t="n"/>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="17" t="n">
         <v>46412</v>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -701,7 +711,7 @@
       <c r="K9" s="7" t="n"/>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="17" t="n">
         <v>46426</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -720,7 +730,7 @@
       <c r="K10" s="7" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="17" t="n">
         <v>46440</v>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -855,7 +865,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="n"/>
+      <c r="A5" s="18" t="n"/>
       <c r="B5" s="15" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -864,7 +874,7 @@
       <c r="G5" s="15" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n"/>
+      <c r="A6" s="18" t="n"/>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -873,7 +883,7 @@
       <c r="G6" s="15" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n"/>
+      <c r="A7" s="18" t="n"/>
       <c r="B7" s="15" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -882,7 +892,7 @@
       <c r="G7" s="15" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n"/>
+      <c r="A8" s="18" t="n"/>
       <c r="B8" s="15" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -891,7 +901,7 @@
       <c r="G8" s="15" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="n"/>
+      <c r="A9" s="18" t="n"/>
       <c r="B9" s="15" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -900,7 +910,7 @@
       <c r="G9" s="15" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="n"/>
+      <c r="A10" s="18" t="n"/>
       <c r="B10" s="15" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -909,7 +919,7 @@
       <c r="G10" s="15" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="n"/>
+      <c r="A11" s="18" t="n"/>
       <c r="B11" s="15" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -918,7 +928,7 @@
       <c r="G11" s="15" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="n"/>
+      <c r="A12" s="18" t="n"/>
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -927,7 +937,7 @@
       <c r="G12" s="15" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="n"/>
+      <c r="A13" s="18" t="n"/>
       <c r="B13" s="15" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -936,7 +946,7 @@
       <c r="G13" s="15" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="n"/>
+      <c r="A14" s="18" t="n"/>
       <c r="B14" s="15" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -945,7 +955,7 @@
       <c r="G14" s="15" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="n"/>
+      <c r="A15" s="18" t="n"/>
       <c r="B15" s="15" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -954,7 +964,7 @@
       <c r="G15" s="15" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n"/>
+      <c r="A16" s="18" t="n"/>
       <c r="B16" s="15" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -963,7 +973,7 @@
       <c r="G16" s="15" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="n"/>
+      <c r="A17" s="18" t="n"/>
       <c r="B17" s="15" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -972,7 +982,7 @@
       <c r="G17" s="15" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="n"/>
+      <c r="A18" s="18" t="n"/>
       <c r="B18" s="15" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
@@ -981,7 +991,7 @@
       <c r="G18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="n"/>
+      <c r="A19" s="18" t="n"/>
       <c r="B19" s="15" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="15" t="n"/>
@@ -990,7 +1000,7 @@
       <c r="G19" s="15" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="n"/>
+      <c r="A20" s="18" t="n"/>
       <c r="B20" s="15" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
@@ -999,7 +1009,7 @@
       <c r="G20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="n"/>
+      <c r="A21" s="18" t="n"/>
       <c r="B21" s="15" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -1008,7 +1018,7 @@
       <c r="G21" s="15" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="n"/>
+      <c r="A22" s="18" t="n"/>
       <c r="B22" s="15" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -1017,7 +1027,7 @@
       <c r="G22" s="15" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="n"/>
+      <c r="A23" s="18" t="n"/>
       <c r="B23" s="15" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -1026,7 +1036,7 @@
       <c r="G23" s="15" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="n"/>
+      <c r="A24" s="18" t="n"/>
       <c r="B24" s="15" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -1035,7 +1045,7 @@
       <c r="G24" s="15" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="n"/>
+      <c r="A25" s="18" t="n"/>
       <c r="B25" s="15" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -1044,7 +1054,7 @@
       <c r="G25" s="15" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="n"/>
+      <c r="A26" s="18" t="n"/>
       <c r="B26" s="15" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -1053,7 +1063,7 @@
       <c r="G26" s="15" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="n"/>
+      <c r="A27" s="18" t="n"/>
       <c r="B27" s="15" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
@@ -1062,7 +1072,7 @@
       <c r="G27" s="15" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="n"/>
+      <c r="A28" s="18" t="n"/>
       <c r="B28" s="15" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -1071,7 +1081,7 @@
       <c r="G28" s="15" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="n"/>
+      <c r="A29" s="18" t="n"/>
       <c r="B29" s="15" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -1080,7 +1090,7 @@
       <c r="G29" s="15" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n"/>
+      <c r="A30" s="18" t="n"/>
       <c r="B30" s="15" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
@@ -1089,7 +1099,7 @@
       <c r="G30" s="15" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="n"/>
+      <c r="A31" s="18" t="n"/>
       <c r="B31" s="15" t="n"/>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
@@ -1098,7 +1108,7 @@
       <c r="G31" s="15" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="n"/>
+      <c r="A32" s="18" t="n"/>
       <c r="B32" s="15" t="n"/>
       <c r="C32" s="15" t="n"/>
       <c r="D32" s="15" t="n"/>
@@ -1107,7 +1117,7 @@
       <c r="G32" s="15" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="n"/>
+      <c r="A33" s="18" t="n"/>
       <c r="B33" s="15" t="n"/>
       <c r="C33" s="15" t="n"/>
       <c r="D33" s="15" t="n"/>
@@ -1116,7 +1126,7 @@
       <c r="G33" s="15" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="n"/>
+      <c r="A34" s="18" t="n"/>
       <c r="B34" s="15" t="n"/>
       <c r="C34" s="15" t="n"/>
       <c r="D34" s="15" t="n"/>
@@ -1125,7 +1135,7 @@
       <c r="G34" s="15" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="n"/>
+      <c r="A35" s="18" t="n"/>
       <c r="B35" s="15" t="n"/>
       <c r="C35" s="15" t="n"/>
       <c r="D35" s="15" t="n"/>
@@ -1134,7 +1144,7 @@
       <c r="G35" s="15" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
+      <c r="A36" s="18" t="n"/>
       <c r="B36" s="15" t="n"/>
       <c r="C36" s="15" t="n"/>
       <c r="D36" s="15" t="n"/>
@@ -1143,7 +1153,7 @@
       <c r="G36" s="15" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
+      <c r="A37" s="18" t="n"/>
       <c r="B37" s="15" t="n"/>
       <c r="C37" s="15" t="n"/>
       <c r="D37" s="15" t="n"/>
@@ -1152,7 +1162,7 @@
       <c r="G37" s="15" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
+      <c r="A38" s="18" t="n"/>
       <c r="B38" s="15" t="n"/>
       <c r="C38" s="15" t="n"/>
       <c r="D38" s="15" t="n"/>
@@ -1161,7 +1171,7 @@
       <c r="G38" s="15" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
+      <c r="A39" s="18" t="n"/>
       <c r="B39" s="15" t="n"/>
       <c r="C39" s="15" t="n"/>
       <c r="D39" s="15" t="n"/>
@@ -1170,7 +1180,7 @@
       <c r="G39" s="15" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="n"/>
+      <c r="A40" s="18" t="n"/>
       <c r="B40" s="15" t="n"/>
       <c r="C40" s="15" t="n"/>
       <c r="D40" s="15" t="n"/>
@@ -1179,7 +1189,7 @@
       <c r="G40" s="15" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
+      <c r="A41" s="18" t="n"/>
       <c r="B41" s="15" t="n"/>
       <c r="C41" s="15" t="n"/>
       <c r="D41" s="15" t="n"/>
@@ -1188,7 +1198,7 @@
       <c r="G41" s="15" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="n"/>
+      <c r="A42" s="18" t="n"/>
       <c r="B42" s="15" t="n"/>
       <c r="C42" s="15" t="n"/>
       <c r="D42" s="15" t="n"/>
@@ -1197,7 +1207,7 @@
       <c r="G42" s="15" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="n"/>
+      <c r="A43" s="18" t="n"/>
       <c r="B43" s="15" t="n"/>
       <c r="C43" s="15" t="n"/>
       <c r="D43" s="15" t="n"/>
@@ -1206,7 +1216,7 @@
       <c r="G43" s="15" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="14" t="n"/>
+      <c r="A44" s="18" t="n"/>
       <c r="B44" s="15" t="n"/>
       <c r="C44" s="15" t="n"/>
       <c r="D44" s="15" t="n"/>
@@ -1215,7 +1225,7 @@
       <c r="G44" s="15" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="n"/>
+      <c r="A45" s="18" t="n"/>
       <c r="B45" s="15" t="n"/>
       <c r="C45" s="15" t="n"/>
       <c r="D45" s="15" t="n"/>
@@ -1224,7 +1234,7 @@
       <c r="G45" s="15" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="n"/>
+      <c r="A46" s="18" t="n"/>
       <c r="B46" s="15" t="n"/>
       <c r="C46" s="15" t="n"/>
       <c r="D46" s="15" t="n"/>
@@ -1233,7 +1243,7 @@
       <c r="G46" s="15" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="n"/>
+      <c r="A47" s="18" t="n"/>
       <c r="B47" s="15" t="n"/>
       <c r="C47" s="15" t="n"/>
       <c r="D47" s="15" t="n"/>
@@ -1242,7 +1252,7 @@
       <c r="G47" s="15" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="n"/>
+      <c r="A48" s="18" t="n"/>
       <c r="B48" s="15" t="n"/>
       <c r="C48" s="15" t="n"/>
       <c r="D48" s="15" t="n"/>
@@ -1251,7 +1261,7 @@
       <c r="G48" s="15" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="14" t="n"/>
+      <c r="A49" s="18" t="n"/>
       <c r="B49" s="15" t="n"/>
       <c r="C49" s="15" t="n"/>
       <c r="D49" s="15" t="n"/>
@@ -1260,7 +1270,7 @@
       <c r="G49" s="15" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="n"/>
+      <c r="A50" s="18" t="n"/>
       <c r="B50" s="15" t="n"/>
       <c r="C50" s="15" t="n"/>
       <c r="D50" s="15" t="n"/>
@@ -1269,7 +1279,7 @@
       <c r="G50" s="15" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="14" t="n"/>
+      <c r="A51" s="18" t="n"/>
       <c r="B51" s="15" t="n"/>
       <c r="C51" s="15" t="n"/>
       <c r="D51" s="15" t="n"/>
@@ -1278,7 +1288,7 @@
       <c r="G51" s="15" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="n"/>
+      <c r="A52" s="18" t="n"/>
       <c r="B52" s="15" t="n"/>
       <c r="C52" s="15" t="n"/>
       <c r="D52" s="15" t="n"/>
@@ -1287,7 +1297,7 @@
       <c r="G52" s="15" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="n"/>
+      <c r="A53" s="18" t="n"/>
       <c r="B53" s="15" t="n"/>
       <c r="C53" s="15" t="n"/>
       <c r="D53" s="15" t="n"/>
@@ -1296,7 +1306,7 @@
       <c r="G53" s="15" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="n"/>
+      <c r="A54" s="18" t="n"/>
       <c r="B54" s="15" t="n"/>
       <c r="C54" s="15" t="n"/>
       <c r="D54" s="15" t="n"/>
@@ -1305,7 +1315,7 @@
       <c r="G54" s="15" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="n"/>
+      <c r="A55" s="18" t="n"/>
       <c r="B55" s="15" t="n"/>
       <c r="C55" s="15" t="n"/>
       <c r="D55" s="15" t="n"/>
@@ -1314,7 +1324,7 @@
       <c r="G55" s="15" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="n"/>
+      <c r="A56" s="18" t="n"/>
       <c r="B56" s="15" t="n"/>
       <c r="C56" s="15" t="n"/>
       <c r="D56" s="15" t="n"/>
@@ -1323,7 +1333,7 @@
       <c r="G56" s="15" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="n"/>
+      <c r="A57" s="18" t="n"/>
       <c r="B57" s="15" t="n"/>
       <c r="C57" s="15" t="n"/>
       <c r="D57" s="15" t="n"/>
@@ -1332,7 +1342,7 @@
       <c r="G57" s="15" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="n"/>
+      <c r="A58" s="18" t="n"/>
       <c r="B58" s="15" t="n"/>
       <c r="C58" s="15" t="n"/>
       <c r="D58" s="15" t="n"/>
@@ -1341,7 +1351,7 @@
       <c r="G58" s="15" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="14" t="n"/>
+      <c r="A59" s="18" t="n"/>
       <c r="B59" s="15" t="n"/>
       <c r="C59" s="15" t="n"/>
       <c r="D59" s="15" t="n"/>
@@ -1350,7 +1360,7 @@
       <c r="G59" s="15" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="14" t="n"/>
+      <c r="A60" s="18" t="n"/>
       <c r="B60" s="15" t="n"/>
       <c r="C60" s="15" t="n"/>
       <c r="D60" s="15" t="n"/>
@@ -1359,7 +1369,7 @@
       <c r="G60" s="15" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="n"/>
+      <c r="A61" s="18" t="n"/>
       <c r="B61" s="15" t="n"/>
       <c r="C61" s="15" t="n"/>
       <c r="D61" s="15" t="n"/>
@@ -1368,7 +1378,7 @@
       <c r="G61" s="15" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="n"/>
+      <c r="A62" s="18" t="n"/>
       <c r="B62" s="15" t="n"/>
       <c r="C62" s="15" t="n"/>
       <c r="D62" s="15" t="n"/>
@@ -1377,7 +1387,7 @@
       <c r="G62" s="15" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="n"/>
+      <c r="A63" s="18" t="n"/>
       <c r="B63" s="15" t="n"/>
       <c r="C63" s="15" t="n"/>
       <c r="D63" s="15" t="n"/>
@@ -1386,7 +1396,7 @@
       <c r="G63" s="15" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="n"/>
+      <c r="A64" s="18" t="n"/>
       <c r="B64" s="15" t="n"/>
       <c r="C64" s="15" t="n"/>
       <c r="D64" s="15" t="n"/>
@@ -1395,7 +1405,7 @@
       <c r="G64" s="15" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="n"/>
+      <c r="A65" s="18" t="n"/>
       <c r="B65" s="15" t="n"/>
       <c r="C65" s="15" t="n"/>
       <c r="D65" s="15" t="n"/>
@@ -1404,7 +1414,7 @@
       <c r="G65" s="15" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="14" t="n"/>
+      <c r="A66" s="18" t="n"/>
       <c r="B66" s="15" t="n"/>
       <c r="C66" s="15" t="n"/>
       <c r="D66" s="15" t="n"/>
@@ -1413,7 +1423,7 @@
       <c r="G66" s="15" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="14" t="n"/>
+      <c r="A67" s="18" t="n"/>
       <c r="B67" s="15" t="n"/>
       <c r="C67" s="15" t="n"/>
       <c r="D67" s="15" t="n"/>
@@ -1422,7 +1432,7 @@
       <c r="G67" s="15" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="14" t="n"/>
+      <c r="A68" s="18" t="n"/>
       <c r="B68" s="15" t="n"/>
       <c r="C68" s="15" t="n"/>
       <c r="D68" s="15" t="n"/>
@@ -1431,7 +1441,7 @@
       <c r="G68" s="15" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="n"/>
+      <c r="A69" s="18" t="n"/>
       <c r="B69" s="15" t="n"/>
       <c r="C69" s="15" t="n"/>
       <c r="D69" s="15" t="n"/>
@@ -1440,7 +1450,7 @@
       <c r="G69" s="15" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="14" t="n"/>
+      <c r="A70" s="18" t="n"/>
       <c r="B70" s="15" t="n"/>
       <c r="C70" s="15" t="n"/>
       <c r="D70" s="15" t="n"/>
@@ -1449,7 +1459,7 @@
       <c r="G70" s="15" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="14" t="n"/>
+      <c r="A71" s="18" t="n"/>
       <c r="B71" s="15" t="n"/>
       <c r="C71" s="15" t="n"/>
       <c r="D71" s="15" t="n"/>
@@ -1458,7 +1468,7 @@
       <c r="G71" s="15" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="14" t="n"/>
+      <c r="A72" s="18" t="n"/>
       <c r="B72" s="15" t="n"/>
       <c r="C72" s="15" t="n"/>
       <c r="D72" s="15" t="n"/>
@@ -1467,7 +1477,7 @@
       <c r="G72" s="15" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="14" t="n"/>
+      <c r="A73" s="18" t="n"/>
       <c r="B73" s="15" t="n"/>
       <c r="C73" s="15" t="n"/>
       <c r="D73" s="15" t="n"/>
@@ -1476,7 +1486,7 @@
       <c r="G73" s="15" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="n"/>
+      <c r="A74" s="18" t="n"/>
       <c r="B74" s="15" t="n"/>
       <c r="C74" s="15" t="n"/>
       <c r="D74" s="15" t="n"/>
@@ -1485,7 +1495,7 @@
       <c r="G74" s="15" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="14" t="n"/>
+      <c r="A75" s="18" t="n"/>
       <c r="B75" s="15" t="n"/>
       <c r="C75" s="15" t="n"/>
       <c r="D75" s="15" t="n"/>
@@ -1494,7 +1504,7 @@
       <c r="G75" s="15" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="n"/>
+      <c r="A76" s="18" t="n"/>
       <c r="B76" s="15" t="n"/>
       <c r="C76" s="15" t="n"/>
       <c r="D76" s="15" t="n"/>
@@ -1503,7 +1513,7 @@
       <c r="G76" s="15" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="14" t="n"/>
+      <c r="A77" s="18" t="n"/>
       <c r="B77" s="15" t="n"/>
       <c r="C77" s="15" t="n"/>
       <c r="D77" s="15" t="n"/>
@@ -1512,7 +1522,7 @@
       <c r="G77" s="15" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="14" t="n"/>
+      <c r="A78" s="18" t="n"/>
       <c r="B78" s="15" t="n"/>
       <c r="C78" s="15" t="n"/>
       <c r="D78" s="15" t="n"/>
@@ -1521,7 +1531,7 @@
       <c r="G78" s="15" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="n"/>
+      <c r="A79" s="18" t="n"/>
       <c r="B79" s="15" t="n"/>
       <c r="C79" s="15" t="n"/>
       <c r="D79" s="15" t="n"/>
@@ -1530,7 +1540,7 @@
       <c r="G79" s="15" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="14" t="n"/>
+      <c r="A80" s="18" t="n"/>
       <c r="B80" s="15" t="n"/>
       <c r="C80" s="15" t="n"/>
       <c r="D80" s="15" t="n"/>
@@ -1539,7 +1549,7 @@
       <c r="G80" s="15" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="14" t="n"/>
+      <c r="A81" s="18" t="n"/>
       <c r="B81" s="15" t="n"/>
       <c r="C81" s="15" t="n"/>
       <c r="D81" s="15" t="n"/>
@@ -1548,7 +1558,7 @@
       <c r="G81" s="15" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="n"/>
+      <c r="A82" s="18" t="n"/>
       <c r="B82" s="15" t="n"/>
       <c r="C82" s="15" t="n"/>
       <c r="D82" s="15" t="n"/>
@@ -1557,7 +1567,7 @@
       <c r="G82" s="15" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="14" t="n"/>
+      <c r="A83" s="18" t="n"/>
       <c r="B83" s="15" t="n"/>
       <c r="C83" s="15" t="n"/>
       <c r="D83" s="15" t="n"/>
@@ -1566,7 +1576,7 @@
       <c r="G83" s="15" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="n"/>
+      <c r="A84" s="18" t="n"/>
       <c r="B84" s="15" t="n"/>
       <c r="C84" s="15" t="n"/>
       <c r="D84" s="15" t="n"/>
@@ -1575,7 +1585,7 @@
       <c r="G84" s="15" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="n"/>
+      <c r="A85" s="18" t="n"/>
       <c r="B85" s="15" t="n"/>
       <c r="C85" s="15" t="n"/>
       <c r="D85" s="15" t="n"/>
@@ -1584,7 +1594,7 @@
       <c r="G85" s="15" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="14" t="n"/>
+      <c r="A86" s="18" t="n"/>
       <c r="B86" s="15" t="n"/>
       <c r="C86" s="15" t="n"/>
       <c r="D86" s="15" t="n"/>
@@ -1593,7 +1603,7 @@
       <c r="G86" s="15" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="14" t="n"/>
+      <c r="A87" s="18" t="n"/>
       <c r="B87" s="15" t="n"/>
       <c r="C87" s="15" t="n"/>
       <c r="D87" s="15" t="n"/>
@@ -1602,7 +1612,7 @@
       <c r="G87" s="15" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="14" t="n"/>
+      <c r="A88" s="18" t="n"/>
       <c r="B88" s="15" t="n"/>
       <c r="C88" s="15" t="n"/>
       <c r="D88" s="15" t="n"/>
@@ -1611,7 +1621,7 @@
       <c r="G88" s="15" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="14" t="n"/>
+      <c r="A89" s="18" t="n"/>
       <c r="B89" s="15" t="n"/>
       <c r="C89" s="15" t="n"/>
       <c r="D89" s="15" t="n"/>
@@ -1620,7 +1630,7 @@
       <c r="G89" s="15" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="n"/>
+      <c r="A90" s="18" t="n"/>
       <c r="B90" s="15" t="n"/>
       <c r="C90" s="15" t="n"/>
       <c r="D90" s="15" t="n"/>
@@ -1629,7 +1639,7 @@
       <c r="G90" s="15" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="n"/>
+      <c r="A91" s="18" t="n"/>
       <c r="B91" s="15" t="n"/>
       <c r="C91" s="15" t="n"/>
       <c r="D91" s="15" t="n"/>
@@ -1638,7 +1648,7 @@
       <c r="G91" s="15" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="14" t="n"/>
+      <c r="A92" s="18" t="n"/>
       <c r="B92" s="15" t="n"/>
       <c r="C92" s="15" t="n"/>
       <c r="D92" s="15" t="n"/>
@@ -1647,7 +1657,7 @@
       <c r="G92" s="15" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="n"/>
+      <c r="A93" s="18" t="n"/>
       <c r="B93" s="15" t="n"/>
       <c r="C93" s="15" t="n"/>
       <c r="D93" s="15" t="n"/>
@@ -1656,7 +1666,7 @@
       <c r="G93" s="15" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="n"/>
+      <c r="A94" s="18" t="n"/>
       <c r="B94" s="15" t="n"/>
       <c r="C94" s="15" t="n"/>
       <c r="D94" s="15" t="n"/>
@@ -1665,7 +1675,7 @@
       <c r="G94" s="15" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="14" t="n"/>
+      <c r="A95" s="18" t="n"/>
       <c r="B95" s="15" t="n"/>
       <c r="C95" s="15" t="n"/>
       <c r="D95" s="15" t="n"/>
@@ -1674,7 +1684,7 @@
       <c r="G95" s="15" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="n"/>
+      <c r="A96" s="18" t="n"/>
       <c r="B96" s="15" t="n"/>
       <c r="C96" s="15" t="n"/>
       <c r="D96" s="15" t="n"/>
@@ -1683,7 +1693,7 @@
       <c r="G96" s="15" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="n"/>
+      <c r="A97" s="18" t="n"/>
       <c r="B97" s="15" t="n"/>
       <c r="C97" s="15" t="n"/>
       <c r="D97" s="15" t="n"/>
@@ -1692,7 +1702,7 @@
       <c r="G97" s="15" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="n"/>
+      <c r="A98" s="18" t="n"/>
       <c r="B98" s="15" t="n"/>
       <c r="C98" s="15" t="n"/>
       <c r="D98" s="15" t="n"/>
@@ -1701,7 +1711,7 @@
       <c r="G98" s="15" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="n"/>
+      <c r="A99" s="18" t="n"/>
       <c r="B99" s="15" t="n"/>
       <c r="C99" s="15" t="n"/>
       <c r="D99" s="15" t="n"/>
@@ -1710,7 +1720,7 @@
       <c r="G99" s="15" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="14" t="n"/>
+      <c r="A100" s="18" t="n"/>
       <c r="B100" s="15" t="n"/>
       <c r="C100" s="15" t="n"/>
       <c r="D100" s="15" t="n"/>
@@ -1719,7 +1729,7 @@
       <c r="G100" s="15" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="14" t="n"/>
+      <c r="A101" s="18" t="n"/>
       <c r="B101" s="15" t="n"/>
       <c r="C101" s="15" t="n"/>
       <c r="D101" s="15" t="n"/>
@@ -1728,7 +1738,7 @@
       <c r="G101" s="15" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="14" t="n"/>
+      <c r="A102" s="18" t="n"/>
       <c r="B102" s="15" t="n"/>
       <c r="C102" s="15" t="n"/>
       <c r="D102" s="15" t="n"/>
@@ -1737,7 +1747,7 @@
       <c r="G102" s="15" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="14" t="n"/>
+      <c r="A103" s="18" t="n"/>
       <c r="B103" s="15" t="n"/>
       <c r="C103" s="15" t="n"/>
       <c r="D103" s="15" t="n"/>
@@ -1746,7 +1756,7 @@
       <c r="G103" s="15" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="n"/>
+      <c r="A104" s="18" t="n"/>
       <c r="B104" s="15" t="n"/>
       <c r="C104" s="15" t="n"/>
       <c r="D104" s="15" t="n"/>
@@ -1755,7 +1765,7 @@
       <c r="G104" s="15" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="14" t="n"/>
+      <c r="A105" s="18" t="n"/>
       <c r="B105" s="15" t="n"/>
       <c r="C105" s="15" t="n"/>
       <c r="D105" s="15" t="n"/>
@@ -1764,7 +1774,7 @@
       <c r="G105" s="15" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="14" t="n"/>
+      <c r="A106" s="18" t="n"/>
       <c r="B106" s="15" t="n"/>
       <c r="C106" s="15" t="n"/>
       <c r="D106" s="15" t="n"/>
@@ -1773,7 +1783,7 @@
       <c r="G106" s="15" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="14" t="n"/>
+      <c r="A107" s="18" t="n"/>
       <c r="B107" s="15" t="n"/>
       <c r="C107" s="15" t="n"/>
       <c r="D107" s="15" t="n"/>
@@ -1782,7 +1792,7 @@
       <c r="G107" s="15" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="14" t="n"/>
+      <c r="A108" s="18" t="n"/>
       <c r="B108" s="15" t="n"/>
       <c r="C108" s="15" t="n"/>
       <c r="D108" s="15" t="n"/>
@@ -1791,7 +1801,7 @@
       <c r="G108" s="15" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="14" t="n"/>
+      <c r="A109" s="18" t="n"/>
       <c r="B109" s="15" t="n"/>
       <c r="C109" s="15" t="n"/>
       <c r="D109" s="15" t="n"/>
@@ -1800,7 +1810,7 @@
       <c r="G109" s="15" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="14" t="n"/>
+      <c r="A110" s="18" t="n"/>
       <c r="B110" s="15" t="n"/>
       <c r="C110" s="15" t="n"/>
       <c r="D110" s="15" t="n"/>
@@ -1809,7 +1819,7 @@
       <c r="G110" s="15" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="14" t="n"/>
+      <c r="A111" s="18" t="n"/>
       <c r="B111" s="15" t="n"/>
       <c r="C111" s="15" t="n"/>
       <c r="D111" s="15" t="n"/>
@@ -1818,7 +1828,7 @@
       <c r="G111" s="15" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="14" t="n"/>
+      <c r="A112" s="18" t="n"/>
       <c r="B112" s="15" t="n"/>
       <c r="C112" s="15" t="n"/>
       <c r="D112" s="15" t="n"/>
@@ -1827,7 +1837,7 @@
       <c r="G112" s="15" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="14" t="n"/>
+      <c r="A113" s="18" t="n"/>
       <c r="B113" s="15" t="n"/>
       <c r="C113" s="15" t="n"/>
       <c r="D113" s="15" t="n"/>
@@ -1836,7 +1846,7 @@
       <c r="G113" s="15" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="14" t="n"/>
+      <c r="A114" s="18" t="n"/>
       <c r="B114" s="15" t="n"/>
       <c r="C114" s="15" t="n"/>
       <c r="D114" s="15" t="n"/>
@@ -1845,7 +1855,7 @@
       <c r="G114" s="15" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="14" t="n"/>
+      <c r="A115" s="18" t="n"/>
       <c r="B115" s="15" t="n"/>
       <c r="C115" s="15" t="n"/>
       <c r="D115" s="15" t="n"/>
@@ -1854,7 +1864,7 @@
       <c r="G115" s="15" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="14" t="n"/>
+      <c r="A116" s="18" t="n"/>
       <c r="B116" s="15" t="n"/>
       <c r="C116" s="15" t="n"/>
       <c r="D116" s="15" t="n"/>
@@ -1863,7 +1873,7 @@
       <c r="G116" s="15" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="14" t="n"/>
+      <c r="A117" s="18" t="n"/>
       <c r="B117" s="15" t="n"/>
       <c r="C117" s="15" t="n"/>
       <c r="D117" s="15" t="n"/>
@@ -1872,7 +1882,7 @@
       <c r="G117" s="15" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="14" t="n"/>
+      <c r="A118" s="18" t="n"/>
       <c r="B118" s="15" t="n"/>
       <c r="C118" s="15" t="n"/>
       <c r="D118" s="15" t="n"/>
@@ -1881,7 +1891,7 @@
       <c r="G118" s="15" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="14" t="n"/>
+      <c r="A119" s="18" t="n"/>
       <c r="B119" s="15" t="n"/>
       <c r="C119" s="15" t="n"/>
       <c r="D119" s="15" t="n"/>
@@ -1890,7 +1900,7 @@
       <c r="G119" s="15" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="14" t="n"/>
+      <c r="A120" s="18" t="n"/>
       <c r="B120" s="15" t="n"/>
       <c r="C120" s="15" t="n"/>
       <c r="D120" s="15" t="n"/>
@@ -1899,7 +1909,7 @@
       <c r="G120" s="15" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="14" t="n"/>
+      <c r="A121" s="18" t="n"/>
       <c r="B121" s="15" t="n"/>
       <c r="C121" s="15" t="n"/>
       <c r="D121" s="15" t="n"/>
@@ -1908,7 +1918,7 @@
       <c r="G121" s="15" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="14" t="n"/>
+      <c r="A122" s="18" t="n"/>
       <c r="B122" s="15" t="n"/>
       <c r="C122" s="15" t="n"/>
       <c r="D122" s="15" t="n"/>
@@ -1917,7 +1927,7 @@
       <c r="G122" s="15" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="14" t="n"/>
+      <c r="A123" s="18" t="n"/>
       <c r="B123" s="15" t="n"/>
       <c r="C123" s="15" t="n"/>
       <c r="D123" s="15" t="n"/>
@@ -1926,7 +1936,7 @@
       <c r="G123" s="15" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="14" t="n"/>
+      <c r="A124" s="18" t="n"/>
       <c r="B124" s="15" t="n"/>
       <c r="C124" s="15" t="n"/>
       <c r="D124" s="15" t="n"/>
@@ -1935,7 +1945,7 @@
       <c r="G124" s="15" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="14" t="n"/>
+      <c r="A125" s="18" t="n"/>
       <c r="B125" s="15" t="n"/>
       <c r="C125" s="15" t="n"/>
       <c r="D125" s="15" t="n"/>
@@ -1944,7 +1954,7 @@
       <c r="G125" s="15" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="14" t="n"/>
+      <c r="A126" s="18" t="n"/>
       <c r="B126" s="15" t="n"/>
       <c r="C126" s="15" t="n"/>
       <c r="D126" s="15" t="n"/>
@@ -1953,7 +1963,7 @@
       <c r="G126" s="15" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="14" t="n"/>
+      <c r="A127" s="18" t="n"/>
       <c r="B127" s="15" t="n"/>
       <c r="C127" s="15" t="n"/>
       <c r="D127" s="15" t="n"/>
@@ -1962,7 +1972,7 @@
       <c r="G127" s="15" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="14" t="n"/>
+      <c r="A128" s="18" t="n"/>
       <c r="B128" s="15" t="n"/>
       <c r="C128" s="15" t="n"/>
       <c r="D128" s="15" t="n"/>
@@ -1971,7 +1981,7 @@
       <c r="G128" s="15" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="14" t="n"/>
+      <c r="A129" s="18" t="n"/>
       <c r="B129" s="15" t="n"/>
       <c r="C129" s="15" t="n"/>
       <c r="D129" s="15" t="n"/>
@@ -1980,7 +1990,7 @@
       <c r="G129" s="15" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="14" t="n"/>
+      <c r="A130" s="18" t="n"/>
       <c r="B130" s="15" t="n"/>
       <c r="C130" s="15" t="n"/>
       <c r="D130" s="15" t="n"/>
@@ -1989,7 +1999,7 @@
       <c r="G130" s="15" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="14" t="n"/>
+      <c r="A131" s="18" t="n"/>
       <c r="B131" s="15" t="n"/>
       <c r="C131" s="15" t="n"/>
       <c r="D131" s="15" t="n"/>
@@ -1998,7 +2008,7 @@
       <c r="G131" s="15" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="14" t="n"/>
+      <c r="A132" s="18" t="n"/>
       <c r="B132" s="15" t="n"/>
       <c r="C132" s="15" t="n"/>
       <c r="D132" s="15" t="n"/>
@@ -2007,7 +2017,7 @@
       <c r="G132" s="15" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="14" t="n"/>
+      <c r="A133" s="18" t="n"/>
       <c r="B133" s="15" t="n"/>
       <c r="C133" s="15" t="n"/>
       <c r="D133" s="15" t="n"/>
@@ -2016,7 +2026,7 @@
       <c r="G133" s="15" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="14" t="n"/>
+      <c r="A134" s="18" t="n"/>
       <c r="B134" s="15" t="n"/>
       <c r="C134" s="15" t="n"/>
       <c r="D134" s="15" t="n"/>
@@ -2025,7 +2035,7 @@
       <c r="G134" s="15" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="14" t="n"/>
+      <c r="A135" s="18" t="n"/>
       <c r="B135" s="15" t="n"/>
       <c r="C135" s="15" t="n"/>
       <c r="D135" s="15" t="n"/>
@@ -2034,7 +2044,7 @@
       <c r="G135" s="15" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="14" t="n"/>
+      <c r="A136" s="18" t="n"/>
       <c r="B136" s="15" t="n"/>
       <c r="C136" s="15" t="n"/>
       <c r="D136" s="15" t="n"/>
@@ -2043,7 +2053,7 @@
       <c r="G136" s="15" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="14" t="n"/>
+      <c r="A137" s="18" t="n"/>
       <c r="B137" s="15" t="n"/>
       <c r="C137" s="15" t="n"/>
       <c r="D137" s="15" t="n"/>
@@ -2052,7 +2062,7 @@
       <c r="G137" s="15" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="14" t="n"/>
+      <c r="A138" s="18" t="n"/>
       <c r="B138" s="15" t="n"/>
       <c r="C138" s="15" t="n"/>
       <c r="D138" s="15" t="n"/>
@@ -2061,7 +2071,7 @@
       <c r="G138" s="15" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="14" t="n"/>
+      <c r="A139" s="18" t="n"/>
       <c r="B139" s="15" t="n"/>
       <c r="C139" s="15" t="n"/>
       <c r="D139" s="15" t="n"/>
@@ -2070,7 +2080,7 @@
       <c r="G139" s="15" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="14" t="n"/>
+      <c r="A140" s="18" t="n"/>
       <c r="B140" s="15" t="n"/>
       <c r="C140" s="15" t="n"/>
       <c r="D140" s="15" t="n"/>
@@ -2079,7 +2089,7 @@
       <c r="G140" s="15" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="14" t="n"/>
+      <c r="A141" s="18" t="n"/>
       <c r="B141" s="15" t="n"/>
       <c r="C141" s="15" t="n"/>
       <c r="D141" s="15" t="n"/>
@@ -2088,7 +2098,7 @@
       <c r="G141" s="15" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="14" t="n"/>
+      <c r="A142" s="18" t="n"/>
       <c r="B142" s="15" t="n"/>
       <c r="C142" s="15" t="n"/>
       <c r="D142" s="15" t="n"/>
@@ -2097,7 +2107,7 @@
       <c r="G142" s="15" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="14" t="n"/>
+      <c r="A143" s="18" t="n"/>
       <c r="B143" s="15" t="n"/>
       <c r="C143" s="15" t="n"/>
       <c r="D143" s="15" t="n"/>
@@ -2106,7 +2116,7 @@
       <c r="G143" s="15" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="14" t="n"/>
+      <c r="A144" s="18" t="n"/>
       <c r="B144" s="15" t="n"/>
       <c r="C144" s="15" t="n"/>
       <c r="D144" s="15" t="n"/>
@@ -2115,7 +2125,7 @@
       <c r="G144" s="15" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="14" t="n"/>
+      <c r="A145" s="18" t="n"/>
       <c r="B145" s="15" t="n"/>
       <c r="C145" s="15" t="n"/>
       <c r="D145" s="15" t="n"/>
@@ -2124,7 +2134,7 @@
       <c r="G145" s="15" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="14" t="n"/>
+      <c r="A146" s="18" t="n"/>
       <c r="B146" s="15" t="n"/>
       <c r="C146" s="15" t="n"/>
       <c r="D146" s="15" t="n"/>
@@ -2133,7 +2143,7 @@
       <c r="G146" s="15" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="14" t="n"/>
+      <c r="A147" s="18" t="n"/>
       <c r="B147" s="15" t="n"/>
       <c r="C147" s="15" t="n"/>
       <c r="D147" s="15" t="n"/>
@@ -2142,7 +2152,7 @@
       <c r="G147" s="15" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="14" t="n"/>
+      <c r="A148" s="18" t="n"/>
       <c r="B148" s="15" t="n"/>
       <c r="C148" s="15" t="n"/>
       <c r="D148" s="15" t="n"/>
@@ -2151,7 +2161,7 @@
       <c r="G148" s="15" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="14" t="n"/>
+      <c r="A149" s="18" t="n"/>
       <c r="B149" s="15" t="n"/>
       <c r="C149" s="15" t="n"/>
       <c r="D149" s="15" t="n"/>
@@ -2160,7 +2170,7 @@
       <c r="G149" s="15" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="14" t="n"/>
+      <c r="A150" s="18" t="n"/>
       <c r="B150" s="15" t="n"/>
       <c r="C150" s="15" t="n"/>
       <c r="D150" s="15" t="n"/>
@@ -2169,7 +2179,7 @@
       <c r="G150" s="15" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="14" t="n"/>
+      <c r="A151" s="18" t="n"/>
       <c r="B151" s="15" t="n"/>
       <c r="C151" s="15" t="n"/>
       <c r="D151" s="15" t="n"/>
@@ -2178,7 +2188,7 @@
       <c r="G151" s="15" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="14" t="n"/>
+      <c r="A152" s="18" t="n"/>
       <c r="B152" s="15" t="n"/>
       <c r="C152" s="15" t="n"/>
       <c r="D152" s="15" t="n"/>
@@ -2187,7 +2197,7 @@
       <c r="G152" s="15" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="14" t="n"/>
+      <c r="A153" s="18" t="n"/>
       <c r="B153" s="15" t="n"/>
       <c r="C153" s="15" t="n"/>
       <c r="D153" s="15" t="n"/>
@@ -2196,7 +2206,7 @@
       <c r="G153" s="15" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="14" t="n"/>
+      <c r="A154" s="18" t="n"/>
       <c r="B154" s="15" t="n"/>
       <c r="C154" s="15" t="n"/>
       <c r="D154" s="15" t="n"/>
@@ -2205,7 +2215,7 @@
       <c r="G154" s="15" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="14" t="n"/>
+      <c r="A155" s="18" t="n"/>
       <c r="B155" s="15" t="n"/>
       <c r="C155" s="15" t="n"/>
       <c r="D155" s="15" t="n"/>
@@ -2214,7 +2224,7 @@
       <c r="G155" s="15" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="14" t="n"/>
+      <c r="A156" s="18" t="n"/>
       <c r="B156" s="15" t="n"/>
       <c r="C156" s="15" t="n"/>
       <c r="D156" s="15" t="n"/>
@@ -2223,7 +2233,7 @@
       <c r="G156" s="15" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="14" t="n"/>
+      <c r="A157" s="18" t="n"/>
       <c r="B157" s="15" t="n"/>
       <c r="C157" s="15" t="n"/>
       <c r="D157" s="15" t="n"/>
@@ -2232,7 +2242,7 @@
       <c r="G157" s="15" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="14" t="n"/>
+      <c r="A158" s="18" t="n"/>
       <c r="B158" s="15" t="n"/>
       <c r="C158" s="15" t="n"/>
       <c r="D158" s="15" t="n"/>
@@ -2241,7 +2251,7 @@
       <c r="G158" s="15" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="14" t="n"/>
+      <c r="A159" s="18" t="n"/>
       <c r="B159" s="15" t="n"/>
       <c r="C159" s="15" t="n"/>
       <c r="D159" s="15" t="n"/>
@@ -2250,7 +2260,7 @@
       <c r="G159" s="15" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="14" t="n"/>
+      <c r="A160" s="18" t="n"/>
       <c r="B160" s="15" t="n"/>
       <c r="C160" s="15" t="n"/>
       <c r="D160" s="15" t="n"/>
@@ -2259,7 +2269,7 @@
       <c r="G160" s="15" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="14" t="n"/>
+      <c r="A161" s="18" t="n"/>
       <c r="B161" s="15" t="n"/>
       <c r="C161" s="15" t="n"/>
       <c r="D161" s="15" t="n"/>
@@ -2268,7 +2278,7 @@
       <c r="G161" s="15" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="14" t="n"/>
+      <c r="A162" s="18" t="n"/>
       <c r="B162" s="15" t="n"/>
       <c r="C162" s="15" t="n"/>
       <c r="D162" s="15" t="n"/>
@@ -2277,7 +2287,7 @@
       <c r="G162" s="15" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="14" t="n"/>
+      <c r="A163" s="18" t="n"/>
       <c r="B163" s="15" t="n"/>
       <c r="C163" s="15" t="n"/>
       <c r="D163" s="15" t="n"/>
@@ -2286,7 +2296,7 @@
       <c r="G163" s="15" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="14" t="n"/>
+      <c r="A164" s="18" t="n"/>
       <c r="B164" s="15" t="n"/>
       <c r="C164" s="15" t="n"/>
       <c r="D164" s="15" t="n"/>
@@ -2295,7 +2305,7 @@
       <c r="G164" s="15" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="14" t="n"/>
+      <c r="A165" s="18" t="n"/>
       <c r="B165" s="15" t="n"/>
       <c r="C165" s="15" t="n"/>
       <c r="D165" s="15" t="n"/>
@@ -2304,7 +2314,7 @@
       <c r="G165" s="15" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="14" t="n"/>
+      <c r="A166" s="18" t="n"/>
       <c r="B166" s="15" t="n"/>
       <c r="C166" s="15" t="n"/>
       <c r="D166" s="15" t="n"/>
@@ -2313,7 +2323,7 @@
       <c r="G166" s="15" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="14" t="n"/>
+      <c r="A167" s="18" t="n"/>
       <c r="B167" s="15" t="n"/>
       <c r="C167" s="15" t="n"/>
       <c r="D167" s="15" t="n"/>
@@ -2322,7 +2332,7 @@
       <c r="G167" s="15" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="14" t="n"/>
+      <c r="A168" s="18" t="n"/>
       <c r="B168" s="15" t="n"/>
       <c r="C168" s="15" t="n"/>
       <c r="D168" s="15" t="n"/>
@@ -2331,7 +2341,7 @@
       <c r="G168" s="15" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="14" t="n"/>
+      <c r="A169" s="18" t="n"/>
       <c r="B169" s="15" t="n"/>
       <c r="C169" s="15" t="n"/>
       <c r="D169" s="15" t="n"/>
@@ -2340,7 +2350,7 @@
       <c r="G169" s="15" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="14" t="n"/>
+      <c r="A170" s="18" t="n"/>
       <c r="B170" s="15" t="n"/>
       <c r="C170" s="15" t="n"/>
       <c r="D170" s="15" t="n"/>
@@ -2349,7 +2359,7 @@
       <c r="G170" s="15" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="14" t="n"/>
+      <c r="A171" s="18" t="n"/>
       <c r="B171" s="15" t="n"/>
       <c r="C171" s="15" t="n"/>
       <c r="D171" s="15" t="n"/>
@@ -2358,7 +2368,7 @@
       <c r="G171" s="15" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="14" t="n"/>
+      <c r="A172" s="18" t="n"/>
       <c r="B172" s="15" t="n"/>
       <c r="C172" s="15" t="n"/>
       <c r="D172" s="15" t="n"/>
@@ -2367,7 +2377,7 @@
       <c r="G172" s="15" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="14" t="n"/>
+      <c r="A173" s="18" t="n"/>
       <c r="B173" s="15" t="n"/>
       <c r="C173" s="15" t="n"/>
       <c r="D173" s="15" t="n"/>
@@ -2376,7 +2386,7 @@
       <c r="G173" s="15" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="14" t="n"/>
+      <c r="A174" s="18" t="n"/>
       <c r="B174" s="15" t="n"/>
       <c r="C174" s="15" t="n"/>
       <c r="D174" s="15" t="n"/>
@@ -2385,7 +2395,7 @@
       <c r="G174" s="15" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="14" t="n"/>
+      <c r="A175" s="18" t="n"/>
       <c r="B175" s="15" t="n"/>
       <c r="C175" s="15" t="n"/>
       <c r="D175" s="15" t="n"/>
@@ -2394,7 +2404,7 @@
       <c r="G175" s="15" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="14" t="n"/>
+      <c r="A176" s="18" t="n"/>
       <c r="B176" s="15" t="n"/>
       <c r="C176" s="15" t="n"/>
       <c r="D176" s="15" t="n"/>
@@ -2403,7 +2413,7 @@
       <c r="G176" s="15" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="14" t="n"/>
+      <c r="A177" s="18" t="n"/>
       <c r="B177" s="15" t="n"/>
       <c r="C177" s="15" t="n"/>
       <c r="D177" s="15" t="n"/>
@@ -2412,7 +2422,7 @@
       <c r="G177" s="15" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="14" t="n"/>
+      <c r="A178" s="18" t="n"/>
       <c r="B178" s="15" t="n"/>
       <c r="C178" s="15" t="n"/>
       <c r="D178" s="15" t="n"/>
@@ -2421,7 +2431,7 @@
       <c r="G178" s="15" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="14" t="n"/>
+      <c r="A179" s="18" t="n"/>
       <c r="B179" s="15" t="n"/>
       <c r="C179" s="15" t="n"/>
       <c r="D179" s="15" t="n"/>
@@ -2430,7 +2440,7 @@
       <c r="G179" s="15" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="14" t="n"/>
+      <c r="A180" s="18" t="n"/>
       <c r="B180" s="15" t="n"/>
       <c r="C180" s="15" t="n"/>
       <c r="D180" s="15" t="n"/>
@@ -2439,7 +2449,7 @@
       <c r="G180" s="15" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="14" t="n"/>
+      <c r="A181" s="18" t="n"/>
       <c r="B181" s="15" t="n"/>
       <c r="C181" s="15" t="n"/>
       <c r="D181" s="15" t="n"/>
@@ -2448,7 +2458,7 @@
       <c r="G181" s="15" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="14" t="n"/>
+      <c r="A182" s="18" t="n"/>
       <c r="B182" s="15" t="n"/>
       <c r="C182" s="15" t="n"/>
       <c r="D182" s="15" t="n"/>
@@ -2457,7 +2467,7 @@
       <c r="G182" s="15" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="14" t="n"/>
+      <c r="A183" s="18" t="n"/>
       <c r="B183" s="15" t="n"/>
       <c r="C183" s="15" t="n"/>
       <c r="D183" s="15" t="n"/>
@@ -2466,7 +2476,7 @@
       <c r="G183" s="15" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="14" t="n"/>
+      <c r="A184" s="18" t="n"/>
       <c r="B184" s="15" t="n"/>
       <c r="C184" s="15" t="n"/>
       <c r="D184" s="15" t="n"/>
@@ -2475,7 +2485,7 @@
       <c r="G184" s="15" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="14" t="n"/>
+      <c r="A185" s="18" t="n"/>
       <c r="B185" s="15" t="n"/>
       <c r="C185" s="15" t="n"/>
       <c r="D185" s="15" t="n"/>
@@ -2484,7 +2494,7 @@
       <c r="G185" s="15" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="14" t="n"/>
+      <c r="A186" s="18" t="n"/>
       <c r="B186" s="15" t="n"/>
       <c r="C186" s="15" t="n"/>
       <c r="D186" s="15" t="n"/>
@@ -2493,7 +2503,7 @@
       <c r="G186" s="15" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="14" t="n"/>
+      <c r="A187" s="18" t="n"/>
       <c r="B187" s="15" t="n"/>
       <c r="C187" s="15" t="n"/>
       <c r="D187" s="15" t="n"/>
@@ -2502,7 +2512,7 @@
       <c r="G187" s="15" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="14" t="n"/>
+      <c r="A188" s="18" t="n"/>
       <c r="B188" s="15" t="n"/>
       <c r="C188" s="15" t="n"/>
       <c r="D188" s="15" t="n"/>
@@ -2511,7 +2521,7 @@
       <c r="G188" s="15" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="14" t="n"/>
+      <c r="A189" s="18" t="n"/>
       <c r="B189" s="15" t="n"/>
       <c r="C189" s="15" t="n"/>
       <c r="D189" s="15" t="n"/>
@@ -2520,7 +2530,7 @@
       <c r="G189" s="15" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="14" t="n"/>
+      <c r="A190" s="18" t="n"/>
       <c r="B190" s="15" t="n"/>
       <c r="C190" s="15" t="n"/>
       <c r="D190" s="15" t="n"/>
@@ -2529,7 +2539,7 @@
       <c r="G190" s="15" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="14" t="n"/>
+      <c r="A191" s="18" t="n"/>
       <c r="B191" s="15" t="n"/>
       <c r="C191" s="15" t="n"/>
       <c r="D191" s="15" t="n"/>
@@ -2538,7 +2548,7 @@
       <c r="G191" s="15" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="14" t="n"/>
+      <c r="A192" s="18" t="n"/>
       <c r="B192" s="15" t="n"/>
       <c r="C192" s="15" t="n"/>
       <c r="D192" s="15" t="n"/>
@@ -2547,7 +2557,7 @@
       <c r="G192" s="15" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="14" t="n"/>
+      <c r="A193" s="18" t="n"/>
       <c r="B193" s="15" t="n"/>
       <c r="C193" s="15" t="n"/>
       <c r="D193" s="15" t="n"/>
@@ -2556,7 +2566,7 @@
       <c r="G193" s="15" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="14" t="n"/>
+      <c r="A194" s="18" t="n"/>
       <c r="B194" s="15" t="n"/>
       <c r="C194" s="15" t="n"/>
       <c r="D194" s="15" t="n"/>
@@ -2565,7 +2575,7 @@
       <c r="G194" s="15" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="14" t="n"/>
+      <c r="A195" s="18" t="n"/>
       <c r="B195" s="15" t="n"/>
       <c r="C195" s="15" t="n"/>
       <c r="D195" s="15" t="n"/>
@@ -2574,7 +2584,7 @@
       <c r="G195" s="15" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="14" t="n"/>
+      <c r="A196" s="18" t="n"/>
       <c r="B196" s="15" t="n"/>
       <c r="C196" s="15" t="n"/>
       <c r="D196" s="15" t="n"/>
@@ -2583,7 +2593,7 @@
       <c r="G196" s="15" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="14" t="n"/>
+      <c r="A197" s="18" t="n"/>
       <c r="B197" s="15" t="n"/>
       <c r="C197" s="15" t="n"/>
       <c r="D197" s="15" t="n"/>
@@ -2592,7 +2602,7 @@
       <c r="G197" s="15" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="14" t="n"/>
+      <c r="A198" s="18" t="n"/>
       <c r="B198" s="15" t="n"/>
       <c r="C198" s="15" t="n"/>
       <c r="D198" s="15" t="n"/>
@@ -2601,7 +2611,7 @@
       <c r="G198" s="15" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="14" t="n"/>
+      <c r="A199" s="18" t="n"/>
       <c r="B199" s="15" t="n"/>
       <c r="C199" s="15" t="n"/>
       <c r="D199" s="15" t="n"/>
@@ -2610,7 +2620,7 @@
       <c r="G199" s="15" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="14" t="n"/>
+      <c r="A200" s="18" t="n"/>
       <c r="B200" s="15" t="n"/>
       <c r="C200" s="15" t="n"/>
       <c r="D200" s="15" t="n"/>
@@ -2619,7 +2629,7 @@
       <c r="G200" s="15" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="14" t="n"/>
+      <c r="A201" s="18" t="n"/>
       <c r="B201" s="15" t="n"/>
       <c r="C201" s="15" t="n"/>
       <c r="D201" s="15" t="n"/>
@@ -2628,7 +2638,7 @@
       <c r="G201" s="15" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="14" t="n"/>
+      <c r="A202" s="18" t="n"/>
       <c r="B202" s="15" t="n"/>
       <c r="C202" s="15" t="n"/>
       <c r="D202" s="15" t="n"/>
@@ -2637,7 +2647,7 @@
       <c r="G202" s="15" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="14" t="n"/>
+      <c r="A203" s="18" t="n"/>
       <c r="B203" s="15" t="n"/>
       <c r="C203" s="15" t="n"/>
       <c r="D203" s="15" t="n"/>
@@ -2646,7 +2656,7 @@
       <c r="G203" s="15" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="14" t="n"/>
+      <c r="A204" s="18" t="n"/>
       <c r="B204" s="15" t="n"/>
       <c r="C204" s="15" t="n"/>
       <c r="D204" s="15" t="n"/>
@@ -2728,700 +2738,700 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="n"/>
+      <c r="A5" s="18" t="n"/>
       <c r="B5" s="15" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="15" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n"/>
+      <c r="A6" s="18" t="n"/>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="15" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n"/>
+      <c r="A7" s="18" t="n"/>
       <c r="B7" s="15" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="15" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n"/>
+      <c r="A8" s="18" t="n"/>
       <c r="B8" s="15" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="15" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="n"/>
+      <c r="A9" s="18" t="n"/>
       <c r="B9" s="15" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="15" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="n"/>
+      <c r="A10" s="18" t="n"/>
       <c r="B10" s="15" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="n"/>
+      <c r="A11" s="18" t="n"/>
       <c r="B11" s="15" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="n"/>
+      <c r="A12" s="18" t="n"/>
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="n"/>
+      <c r="A13" s="18" t="n"/>
       <c r="B13" s="15" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="15" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="n"/>
+      <c r="A14" s="18" t="n"/>
       <c r="B14" s="15" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="n"/>
+      <c r="A15" s="18" t="n"/>
       <c r="B15" s="15" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="15" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n"/>
+      <c r="A16" s="18" t="n"/>
       <c r="B16" s="15" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="15" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="n"/>
+      <c r="A17" s="18" t="n"/>
       <c r="B17" s="15" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="n"/>
+      <c r="A18" s="18" t="n"/>
       <c r="B18" s="15" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="n"/>
+      <c r="A19" s="18" t="n"/>
       <c r="B19" s="15" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="15" t="n"/>
       <c r="E19" s="15" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="n"/>
+      <c r="A20" s="18" t="n"/>
       <c r="B20" s="15" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="n"/>
+      <c r="A21" s="18" t="n"/>
       <c r="B21" s="15" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="15" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="n"/>
+      <c r="A22" s="18" t="n"/>
       <c r="B22" s="15" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="15" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="n"/>
+      <c r="A23" s="18" t="n"/>
       <c r="B23" s="15" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="15" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="n"/>
+      <c r="A24" s="18" t="n"/>
       <c r="B24" s="15" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="15" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="n"/>
+      <c r="A25" s="18" t="n"/>
       <c r="B25" s="15" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="15" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="n"/>
+      <c r="A26" s="18" t="n"/>
       <c r="B26" s="15" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="15" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="n"/>
+      <c r="A27" s="18" t="n"/>
       <c r="B27" s="15" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="15" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="n"/>
+      <c r="A28" s="18" t="n"/>
       <c r="B28" s="15" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="15" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="n"/>
+      <c r="A29" s="18" t="n"/>
       <c r="B29" s="15" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="15" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n"/>
+      <c r="A30" s="18" t="n"/>
       <c r="B30" s="15" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="15" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="n"/>
+      <c r="A31" s="18" t="n"/>
       <c r="B31" s="15" t="n"/>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="15" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="n"/>
+      <c r="A32" s="18" t="n"/>
       <c r="B32" s="15" t="n"/>
       <c r="C32" s="15" t="n"/>
       <c r="D32" s="15" t="n"/>
       <c r="E32" s="15" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="n"/>
+      <c r="A33" s="18" t="n"/>
       <c r="B33" s="15" t="n"/>
       <c r="C33" s="15" t="n"/>
       <c r="D33" s="15" t="n"/>
       <c r="E33" s="15" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="n"/>
+      <c r="A34" s="18" t="n"/>
       <c r="B34" s="15" t="n"/>
       <c r="C34" s="15" t="n"/>
       <c r="D34" s="15" t="n"/>
       <c r="E34" s="15" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="n"/>
+      <c r="A35" s="18" t="n"/>
       <c r="B35" s="15" t="n"/>
       <c r="C35" s="15" t="n"/>
       <c r="D35" s="15" t="n"/>
       <c r="E35" s="15" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
+      <c r="A36" s="18" t="n"/>
       <c r="B36" s="15" t="n"/>
       <c r="C36" s="15" t="n"/>
       <c r="D36" s="15" t="n"/>
       <c r="E36" s="15" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
+      <c r="A37" s="18" t="n"/>
       <c r="B37" s="15" t="n"/>
       <c r="C37" s="15" t="n"/>
       <c r="D37" s="15" t="n"/>
       <c r="E37" s="15" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
+      <c r="A38" s="18" t="n"/>
       <c r="B38" s="15" t="n"/>
       <c r="C38" s="15" t="n"/>
       <c r="D38" s="15" t="n"/>
       <c r="E38" s="15" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
+      <c r="A39" s="18" t="n"/>
       <c r="B39" s="15" t="n"/>
       <c r="C39" s="15" t="n"/>
       <c r="D39" s="15" t="n"/>
       <c r="E39" s="15" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="n"/>
+      <c r="A40" s="18" t="n"/>
       <c r="B40" s="15" t="n"/>
       <c r="C40" s="15" t="n"/>
       <c r="D40" s="15" t="n"/>
       <c r="E40" s="15" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
+      <c r="A41" s="18" t="n"/>
       <c r="B41" s="15" t="n"/>
       <c r="C41" s="15" t="n"/>
       <c r="D41" s="15" t="n"/>
       <c r="E41" s="15" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="n"/>
+      <c r="A42" s="18" t="n"/>
       <c r="B42" s="15" t="n"/>
       <c r="C42" s="15" t="n"/>
       <c r="D42" s="15" t="n"/>
       <c r="E42" s="15" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="n"/>
+      <c r="A43" s="18" t="n"/>
       <c r="B43" s="15" t="n"/>
       <c r="C43" s="15" t="n"/>
       <c r="D43" s="15" t="n"/>
       <c r="E43" s="15" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="14" t="n"/>
+      <c r="A44" s="18" t="n"/>
       <c r="B44" s="15" t="n"/>
       <c r="C44" s="15" t="n"/>
       <c r="D44" s="15" t="n"/>
       <c r="E44" s="15" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="n"/>
+      <c r="A45" s="18" t="n"/>
       <c r="B45" s="15" t="n"/>
       <c r="C45" s="15" t="n"/>
       <c r="D45" s="15" t="n"/>
       <c r="E45" s="15" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="n"/>
+      <c r="A46" s="18" t="n"/>
       <c r="B46" s="15" t="n"/>
       <c r="C46" s="15" t="n"/>
       <c r="D46" s="15" t="n"/>
       <c r="E46" s="15" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="n"/>
+      <c r="A47" s="18" t="n"/>
       <c r="B47" s="15" t="n"/>
       <c r="C47" s="15" t="n"/>
       <c r="D47" s="15" t="n"/>
       <c r="E47" s="15" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="n"/>
+      <c r="A48" s="18" t="n"/>
       <c r="B48" s="15" t="n"/>
       <c r="C48" s="15" t="n"/>
       <c r="D48" s="15" t="n"/>
       <c r="E48" s="15" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="14" t="n"/>
+      <c r="A49" s="18" t="n"/>
       <c r="B49" s="15" t="n"/>
       <c r="C49" s="15" t="n"/>
       <c r="D49" s="15" t="n"/>
       <c r="E49" s="15" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="n"/>
+      <c r="A50" s="18" t="n"/>
       <c r="B50" s="15" t="n"/>
       <c r="C50" s="15" t="n"/>
       <c r="D50" s="15" t="n"/>
       <c r="E50" s="15" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="14" t="n"/>
+      <c r="A51" s="18" t="n"/>
       <c r="B51" s="15" t="n"/>
       <c r="C51" s="15" t="n"/>
       <c r="D51" s="15" t="n"/>
       <c r="E51" s="15" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="n"/>
+      <c r="A52" s="18" t="n"/>
       <c r="B52" s="15" t="n"/>
       <c r="C52" s="15" t="n"/>
       <c r="D52" s="15" t="n"/>
       <c r="E52" s="15" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="n"/>
+      <c r="A53" s="18" t="n"/>
       <c r="B53" s="15" t="n"/>
       <c r="C53" s="15" t="n"/>
       <c r="D53" s="15" t="n"/>
       <c r="E53" s="15" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="n"/>
+      <c r="A54" s="18" t="n"/>
       <c r="B54" s="15" t="n"/>
       <c r="C54" s="15" t="n"/>
       <c r="D54" s="15" t="n"/>
       <c r="E54" s="15" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="n"/>
+      <c r="A55" s="18" t="n"/>
       <c r="B55" s="15" t="n"/>
       <c r="C55" s="15" t="n"/>
       <c r="D55" s="15" t="n"/>
       <c r="E55" s="15" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="n"/>
+      <c r="A56" s="18" t="n"/>
       <c r="B56" s="15" t="n"/>
       <c r="C56" s="15" t="n"/>
       <c r="D56" s="15" t="n"/>
       <c r="E56" s="15" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="n"/>
+      <c r="A57" s="18" t="n"/>
       <c r="B57" s="15" t="n"/>
       <c r="C57" s="15" t="n"/>
       <c r="D57" s="15" t="n"/>
       <c r="E57" s="15" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="n"/>
+      <c r="A58" s="18" t="n"/>
       <c r="B58" s="15" t="n"/>
       <c r="C58" s="15" t="n"/>
       <c r="D58" s="15" t="n"/>
       <c r="E58" s="15" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="14" t="n"/>
+      <c r="A59" s="18" t="n"/>
       <c r="B59" s="15" t="n"/>
       <c r="C59" s="15" t="n"/>
       <c r="D59" s="15" t="n"/>
       <c r="E59" s="15" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="14" t="n"/>
+      <c r="A60" s="18" t="n"/>
       <c r="B60" s="15" t="n"/>
       <c r="C60" s="15" t="n"/>
       <c r="D60" s="15" t="n"/>
       <c r="E60" s="15" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="n"/>
+      <c r="A61" s="18" t="n"/>
       <c r="B61" s="15" t="n"/>
       <c r="C61" s="15" t="n"/>
       <c r="D61" s="15" t="n"/>
       <c r="E61" s="15" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="n"/>
+      <c r="A62" s="18" t="n"/>
       <c r="B62" s="15" t="n"/>
       <c r="C62" s="15" t="n"/>
       <c r="D62" s="15" t="n"/>
       <c r="E62" s="15" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="n"/>
+      <c r="A63" s="18" t="n"/>
       <c r="B63" s="15" t="n"/>
       <c r="C63" s="15" t="n"/>
       <c r="D63" s="15" t="n"/>
       <c r="E63" s="15" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="n"/>
+      <c r="A64" s="18" t="n"/>
       <c r="B64" s="15" t="n"/>
       <c r="C64" s="15" t="n"/>
       <c r="D64" s="15" t="n"/>
       <c r="E64" s="15" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="n"/>
+      <c r="A65" s="18" t="n"/>
       <c r="B65" s="15" t="n"/>
       <c r="C65" s="15" t="n"/>
       <c r="D65" s="15" t="n"/>
       <c r="E65" s="15" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="14" t="n"/>
+      <c r="A66" s="18" t="n"/>
       <c r="B66" s="15" t="n"/>
       <c r="C66" s="15" t="n"/>
       <c r="D66" s="15" t="n"/>
       <c r="E66" s="15" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="14" t="n"/>
+      <c r="A67" s="18" t="n"/>
       <c r="B67" s="15" t="n"/>
       <c r="C67" s="15" t="n"/>
       <c r="D67" s="15" t="n"/>
       <c r="E67" s="15" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="14" t="n"/>
+      <c r="A68" s="18" t="n"/>
       <c r="B68" s="15" t="n"/>
       <c r="C68" s="15" t="n"/>
       <c r="D68" s="15" t="n"/>
       <c r="E68" s="15" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="n"/>
+      <c r="A69" s="18" t="n"/>
       <c r="B69" s="15" t="n"/>
       <c r="C69" s="15" t="n"/>
       <c r="D69" s="15" t="n"/>
       <c r="E69" s="15" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="14" t="n"/>
+      <c r="A70" s="18" t="n"/>
       <c r="B70" s="15" t="n"/>
       <c r="C70" s="15" t="n"/>
       <c r="D70" s="15" t="n"/>
       <c r="E70" s="15" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="14" t="n"/>
+      <c r="A71" s="18" t="n"/>
       <c r="B71" s="15" t="n"/>
       <c r="C71" s="15" t="n"/>
       <c r="D71" s="15" t="n"/>
       <c r="E71" s="15" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="14" t="n"/>
+      <c r="A72" s="18" t="n"/>
       <c r="B72" s="15" t="n"/>
       <c r="C72" s="15" t="n"/>
       <c r="D72" s="15" t="n"/>
       <c r="E72" s="15" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="14" t="n"/>
+      <c r="A73" s="18" t="n"/>
       <c r="B73" s="15" t="n"/>
       <c r="C73" s="15" t="n"/>
       <c r="D73" s="15" t="n"/>
       <c r="E73" s="15" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="n"/>
+      <c r="A74" s="18" t="n"/>
       <c r="B74" s="15" t="n"/>
       <c r="C74" s="15" t="n"/>
       <c r="D74" s="15" t="n"/>
       <c r="E74" s="15" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="14" t="n"/>
+      <c r="A75" s="18" t="n"/>
       <c r="B75" s="15" t="n"/>
       <c r="C75" s="15" t="n"/>
       <c r="D75" s="15" t="n"/>
       <c r="E75" s="15" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="n"/>
+      <c r="A76" s="18" t="n"/>
       <c r="B76" s="15" t="n"/>
       <c r="C76" s="15" t="n"/>
       <c r="D76" s="15" t="n"/>
       <c r="E76" s="15" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="14" t="n"/>
+      <c r="A77" s="18" t="n"/>
       <c r="B77" s="15" t="n"/>
       <c r="C77" s="15" t="n"/>
       <c r="D77" s="15" t="n"/>
       <c r="E77" s="15" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="14" t="n"/>
+      <c r="A78" s="18" t="n"/>
       <c r="B78" s="15" t="n"/>
       <c r="C78" s="15" t="n"/>
       <c r="D78" s="15" t="n"/>
       <c r="E78" s="15" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="n"/>
+      <c r="A79" s="18" t="n"/>
       <c r="B79" s="15" t="n"/>
       <c r="C79" s="15" t="n"/>
       <c r="D79" s="15" t="n"/>
       <c r="E79" s="15" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="14" t="n"/>
+      <c r="A80" s="18" t="n"/>
       <c r="B80" s="15" t="n"/>
       <c r="C80" s="15" t="n"/>
       <c r="D80" s="15" t="n"/>
       <c r="E80" s="15" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="14" t="n"/>
+      <c r="A81" s="18" t="n"/>
       <c r="B81" s="15" t="n"/>
       <c r="C81" s="15" t="n"/>
       <c r="D81" s="15" t="n"/>
       <c r="E81" s="15" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="14" t="n"/>
+      <c r="A82" s="18" t="n"/>
       <c r="B82" s="15" t="n"/>
       <c r="C82" s="15" t="n"/>
       <c r="D82" s="15" t="n"/>
       <c r="E82" s="15" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="14" t="n"/>
+      <c r="A83" s="18" t="n"/>
       <c r="B83" s="15" t="n"/>
       <c r="C83" s="15" t="n"/>
       <c r="D83" s="15" t="n"/>
       <c r="E83" s="15" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="n"/>
+      <c r="A84" s="18" t="n"/>
       <c r="B84" s="15" t="n"/>
       <c r="C84" s="15" t="n"/>
       <c r="D84" s="15" t="n"/>
       <c r="E84" s="15" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="14" t="n"/>
+      <c r="A85" s="18" t="n"/>
       <c r="B85" s="15" t="n"/>
       <c r="C85" s="15" t="n"/>
       <c r="D85" s="15" t="n"/>
       <c r="E85" s="15" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="14" t="n"/>
+      <c r="A86" s="18" t="n"/>
       <c r="B86" s="15" t="n"/>
       <c r="C86" s="15" t="n"/>
       <c r="D86" s="15" t="n"/>
       <c r="E86" s="15" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="14" t="n"/>
+      <c r="A87" s="18" t="n"/>
       <c r="B87" s="15" t="n"/>
       <c r="C87" s="15" t="n"/>
       <c r="D87" s="15" t="n"/>
       <c r="E87" s="15" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="14" t="n"/>
+      <c r="A88" s="18" t="n"/>
       <c r="B88" s="15" t="n"/>
       <c r="C88" s="15" t="n"/>
       <c r="D88" s="15" t="n"/>
       <c r="E88" s="15" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="14" t="n"/>
+      <c r="A89" s="18" t="n"/>
       <c r="B89" s="15" t="n"/>
       <c r="C89" s="15" t="n"/>
       <c r="D89" s="15" t="n"/>
       <c r="E89" s="15" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="n"/>
+      <c r="A90" s="18" t="n"/>
       <c r="B90" s="15" t="n"/>
       <c r="C90" s="15" t="n"/>
       <c r="D90" s="15" t="n"/>
       <c r="E90" s="15" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="n"/>
+      <c r="A91" s="18" t="n"/>
       <c r="B91" s="15" t="n"/>
       <c r="C91" s="15" t="n"/>
       <c r="D91" s="15" t="n"/>
       <c r="E91" s="15" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="14" t="n"/>
+      <c r="A92" s="18" t="n"/>
       <c r="B92" s="15" t="n"/>
       <c r="C92" s="15" t="n"/>
       <c r="D92" s="15" t="n"/>
       <c r="E92" s="15" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="14" t="n"/>
+      <c r="A93" s="18" t="n"/>
       <c r="B93" s="15" t="n"/>
       <c r="C93" s="15" t="n"/>
       <c r="D93" s="15" t="n"/>
       <c r="E93" s="15" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="n"/>
+      <c r="A94" s="18" t="n"/>
       <c r="B94" s="15" t="n"/>
       <c r="C94" s="15" t="n"/>
       <c r="D94" s="15" t="n"/>
       <c r="E94" s="15" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="14" t="n"/>
+      <c r="A95" s="18" t="n"/>
       <c r="B95" s="15" t="n"/>
       <c r="C95" s="15" t="n"/>
       <c r="D95" s="15" t="n"/>
       <c r="E95" s="15" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="n"/>
+      <c r="A96" s="18" t="n"/>
       <c r="B96" s="15" t="n"/>
       <c r="C96" s="15" t="n"/>
       <c r="D96" s="15" t="n"/>
       <c r="E96" s="15" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="14" t="n"/>
+      <c r="A97" s="18" t="n"/>
       <c r="B97" s="15" t="n"/>
       <c r="C97" s="15" t="n"/>
       <c r="D97" s="15" t="n"/>
       <c r="E97" s="15" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="14" t="n"/>
+      <c r="A98" s="18" t="n"/>
       <c r="B98" s="15" t="n"/>
       <c r="C98" s="15" t="n"/>
       <c r="D98" s="15" t="n"/>
       <c r="E98" s="15" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="n"/>
+      <c r="A99" s="18" t="n"/>
       <c r="B99" s="15" t="n"/>
       <c r="C99" s="15" t="n"/>
       <c r="D99" s="15" t="n"/>
       <c r="E99" s="15" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="14" t="n"/>
+      <c r="A100" s="18" t="n"/>
       <c r="B100" s="15" t="n"/>
       <c r="C100" s="15" t="n"/>
       <c r="D100" s="15" t="n"/>
       <c r="E100" s="15" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="14" t="n"/>
+      <c r="A101" s="18" t="n"/>
       <c r="B101" s="15" t="n"/>
       <c r="C101" s="15" t="n"/>
       <c r="D101" s="15" t="n"/>
       <c r="E101" s="15" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="14" t="n"/>
+      <c r="A102" s="18" t="n"/>
       <c r="B102" s="15" t="n"/>
       <c r="C102" s="15" t="n"/>
       <c r="D102" s="15" t="n"/>
       <c r="E102" s="15" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="14" t="n"/>
+      <c r="A103" s="18" t="n"/>
       <c r="B103" s="15" t="n"/>
       <c r="C103" s="15" t="n"/>
       <c r="D103" s="15" t="n"/>
       <c r="E103" s="15" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="n"/>
+      <c r="A104" s="18" t="n"/>
       <c r="B104" s="15" t="n"/>
       <c r="C104" s="15" t="n"/>
       <c r="D104" s="15" t="n"/>

</xml_diff>